<commit_message>
Updated dataset and preprocessing files
</commit_message>
<xml_diff>
--- a/dataset.xlsx
+++ b/dataset.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SAKSHI SHETTY P\Desktop\voxintel_project\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\TANVI\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87B19758-3089-4AAF-863F-66E35617667A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16E487C6-200E-47B8-8248-C9812FA0A55D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2455" uniqueCount="1234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2605" uniqueCount="1293">
   <si>
     <t>tulu_text</t>
   </si>
@@ -3722,6 +3722,183 @@
   </si>
   <si>
     <t>ಈ ಪ್ರಶ್ನೆಲೆನ್ ಎಂಕ್ ಅಭ್ಯಾಸ ಮಲ್ಪೊಡು</t>
+  </si>
+  <si>
+    <t>What day of the week is today</t>
+  </si>
+  <si>
+    <t>ಇನಿ ವಾರದ ವಾ ದಿನ</t>
+  </si>
+  <si>
+    <t>What is today’s full date</t>
+  </si>
+  <si>
+    <t>ಇನಿತ ಪೂರ್ತಿ ದಿನಾಂಕ ದಾದ</t>
+  </si>
+  <si>
+    <t>What day is tomorrow</t>
+  </si>
+  <si>
+    <t>ಎಲ್ಲೆ ದಾದ ದಿನ</t>
+  </si>
+  <si>
+    <t>What day was yesterday</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ಕೋಡೆ ಒವ್ವು ದಿನ </t>
+  </si>
+  <si>
+    <t>What is the date now</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ಇನಿ ಒವ್ವು ದಿನ </t>
+  </si>
+  <si>
+    <t>What is the date this month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ಈ ತಿಂಗೊಲ್ದ ದಿನಾಂಕ ದಾದ </t>
+  </si>
+  <si>
+    <t>Which year is now</t>
+  </si>
+  <si>
+    <t>ಇತ್ತೆ ವಾ ವರ್ಷ</t>
+  </si>
+  <si>
+    <t>Which month is going on</t>
+  </si>
+  <si>
+    <t>ಒವ್ವು ತಿಂಗೊಲ್ ನಡತೊಂದುಂಡು</t>
+  </si>
+  <si>
+    <t>Tell today’s day and date</t>
+  </si>
+  <si>
+    <t>ಇನಿತ  ದಿನ ಬೊಕ್ಕ ದಿನಾಂಕನ್ ಪನ್ಲೆ</t>
+  </si>
+  <si>
+    <t>What is the time and date now</t>
+  </si>
+  <si>
+    <t>ಇತ್ತೆ ಪೊರ್ತು ಬೊಕ್ಕ ದಿನಾಂಕ ದಾದ</t>
+  </si>
+  <si>
+    <t>tomorrow_day</t>
+  </si>
+  <si>
+    <t>yesterday_day</t>
+  </si>
+  <si>
+    <t>Open the window</t>
+  </si>
+  <si>
+    <t>ಕಿಟಕಿನ್ ತೆರೆಲೆ</t>
+  </si>
+  <si>
+    <t>Close the window</t>
+  </si>
+  <si>
+    <t>ಕಿಟಕಿನ್ ಮುಚ್ಚುಲೆ</t>
+  </si>
+  <si>
+    <t>ಬಾಕಿಲ್ ತೆರೆಯೊಡು</t>
+  </si>
+  <si>
+    <t>ಬಾಕಿಲ್ ನ್ ನೂಕುಲೆ</t>
+  </si>
+  <si>
+    <t>ಬಾಕಿಲ್ ನ್ ಒಯಿಪುಲೆ</t>
+  </si>
+  <si>
+    <t>Open the curtain</t>
+  </si>
+  <si>
+    <t>ಪರದೆನ್ ತೆರೆಲೆ</t>
+  </si>
+  <si>
+    <t>Close the curtain</t>
+  </si>
+  <si>
+    <t>ಪರದೆನ್ ಮುಚ್ಚುಲೆ</t>
+  </si>
+  <si>
+    <t>open_gate</t>
+  </si>
+  <si>
+    <t>close_gate</t>
+  </si>
+  <si>
+    <t>open_window</t>
+  </si>
+  <si>
+    <t>close_window</t>
+  </si>
+  <si>
+    <t>open_curtain</t>
+  </si>
+  <si>
+    <t>close_curtain</t>
+  </si>
+  <si>
+    <t>The house is beautiful</t>
+  </si>
+  <si>
+    <t>ಇಲ್ಲ್ ಪೊರ್ಲು ಉಂಡು</t>
+  </si>
+  <si>
+    <t>This road is long</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ಈ ಸಾದಿ ಉದ್ದ ಉಂಡು </t>
+  </si>
+  <si>
+    <t>ಈ  ಪರ್ನ್ದ್ ಚೀಪೆ ಉಂಡು</t>
+  </si>
+  <si>
+    <t>This fruit is sweet</t>
+  </si>
+  <si>
+    <t>That tree is tall</t>
+  </si>
+  <si>
+    <t>This water is cold</t>
+  </si>
+  <si>
+    <t>That room is small</t>
+  </si>
+  <si>
+    <t>This book is interesting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ಆ ಕೋಣೆ ಎಲ್ಯ ಉಂಡು </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ಈ ಪುಸ್ತಕ ಕುತೂಹಲಕಾರಿ ಉಂಡು </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ಈ ನೀರ್ ತಂಪು ಉಂಡು </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ಆ ಮರ ಉದ್ದ ಉಂಡು </t>
+  </si>
+  <si>
+    <t>Our village is peaceful</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ನಮ್ಮ ಊರುಡು ಶಾಂತಿಯುತವಾತ್ ಉಂಡು </t>
+  </si>
+  <si>
+    <t>This flower is nice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ಈ ಪೂ ಪೊರ್ಲು ಉಂಡು </t>
+  </si>
+  <si>
+    <t>That river is deep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ಆ ಸುದೆ ಗುಂಡಿ ಉಂಡು </t>
   </si>
 </sst>
 </file>
@@ -3768,7 +3945,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -3779,7 +3956,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4082,14 +4258,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E491"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <dimension ref="A1:E521"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="53" customWidth="1"/>
-    <col min="2" max="2" width="37.6328125" customWidth="1"/>
-    <col min="3" max="3" width="13.6328125" customWidth="1"/>
-    <col min="4" max="4" width="34.6328125" customWidth="1"/>
-    <col min="5" max="5" width="19.453125" customWidth="1"/>
+    <col min="2" max="2" width="37.6640625" customWidth="1"/>
+    <col min="3" max="3" width="13.6640625" customWidth="1"/>
+    <col min="4" max="4" width="34.6640625" customWidth="1"/>
+    <col min="5" max="5" width="19.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -11946,7 +12122,7 @@
         <v>1161</v>
       </c>
     </row>
-    <row r="463" spans="1:5" ht="15.5">
+    <row r="463" spans="1:5" ht="15">
       <c r="A463" s="3" t="s">
         <v>1206</v>
       </c>
@@ -12151,7 +12327,7 @@
       </c>
     </row>
     <row r="475" spans="1:5">
-      <c r="A475" s="4" t="s">
+      <c r="A475" t="s">
         <v>1217</v>
       </c>
       <c r="B475" t="s">
@@ -12437,6 +12613,516 @@
       </c>
       <c r="E491" t="s">
         <v>1189</v>
+      </c>
+    </row>
+    <row r="492" spans="1:5">
+      <c r="A492" t="s">
+        <v>1235</v>
+      </c>
+      <c r="B492" t="s">
+        <v>1234</v>
+      </c>
+      <c r="C492" t="s">
+        <v>286</v>
+      </c>
+      <c r="D492" t="s">
+        <v>313</v>
+      </c>
+      <c r="E492" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="493" spans="1:5">
+      <c r="A493" t="s">
+        <v>1237</v>
+      </c>
+      <c r="B493" t="s">
+        <v>1236</v>
+      </c>
+      <c r="C493" t="s">
+        <v>286</v>
+      </c>
+      <c r="D493" t="s">
+        <v>305</v>
+      </c>
+      <c r="E493" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="494" spans="1:5">
+      <c r="A494" t="s">
+        <v>1241</v>
+      </c>
+      <c r="B494" t="s">
+        <v>1240</v>
+      </c>
+      <c r="C494" t="s">
+        <v>286</v>
+      </c>
+      <c r="D494" t="s">
+        <v>1254</v>
+      </c>
+      <c r="E494" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="495" spans="1:5">
+      <c r="A495" t="s">
+        <v>1239</v>
+      </c>
+      <c r="B495" s="1" t="s">
+        <v>1238</v>
+      </c>
+      <c r="C495" t="s">
+        <v>286</v>
+      </c>
+      <c r="D495" t="s">
+        <v>1255</v>
+      </c>
+      <c r="E495" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="496" spans="1:5">
+      <c r="A496" t="s">
+        <v>1243</v>
+      </c>
+      <c r="B496" t="s">
+        <v>1242</v>
+      </c>
+      <c r="C496" t="s">
+        <v>286</v>
+      </c>
+      <c r="D496" t="s">
+        <v>305</v>
+      </c>
+      <c r="E496" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="497" spans="1:5">
+      <c r="A497" t="s">
+        <v>1245</v>
+      </c>
+      <c r="B497" t="s">
+        <v>1244</v>
+      </c>
+      <c r="C497" t="s">
+        <v>286</v>
+      </c>
+      <c r="D497" t="s">
+        <v>305</v>
+      </c>
+      <c r="E497" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="498" spans="1:5">
+      <c r="A498" t="s">
+        <v>1247</v>
+      </c>
+      <c r="B498" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C498" t="s">
+        <v>286</v>
+      </c>
+      <c r="D498" t="s">
+        <v>337</v>
+      </c>
+      <c r="E498" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="499" spans="1:5">
+      <c r="A499" t="s">
+        <v>1249</v>
+      </c>
+      <c r="B499" t="s">
+        <v>1248</v>
+      </c>
+      <c r="C499" t="s">
+        <v>286</v>
+      </c>
+      <c r="D499" t="s">
+        <v>340</v>
+      </c>
+      <c r="E499" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="500" spans="1:5">
+      <c r="A500" t="s">
+        <v>1251</v>
+      </c>
+      <c r="B500" t="s">
+        <v>1250</v>
+      </c>
+      <c r="C500" t="s">
+        <v>286</v>
+      </c>
+      <c r="D500" t="s">
+        <v>328</v>
+      </c>
+      <c r="E500" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="501" spans="1:5">
+      <c r="A501" t="s">
+        <v>1253</v>
+      </c>
+      <c r="B501" t="s">
+        <v>1252</v>
+      </c>
+      <c r="C501" t="s">
+        <v>286</v>
+      </c>
+      <c r="D501" t="s">
+        <v>334</v>
+      </c>
+      <c r="E501" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="502" spans="1:5">
+      <c r="A502" t="s">
+        <v>564</v>
+      </c>
+      <c r="B502" t="s">
+        <v>565</v>
+      </c>
+      <c r="C502" t="s">
+        <v>286</v>
+      </c>
+      <c r="D502" t="s">
+        <v>1267</v>
+      </c>
+      <c r="E502" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="503" spans="1:5">
+      <c r="A503" t="s">
+        <v>566</v>
+      </c>
+      <c r="B503" t="s">
+        <v>567</v>
+      </c>
+      <c r="C503" t="s">
+        <v>286</v>
+      </c>
+      <c r="D503" t="s">
+        <v>1268</v>
+      </c>
+      <c r="E503" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="504" spans="1:5">
+      <c r="A504" t="s">
+        <v>1257</v>
+      </c>
+      <c r="B504" t="s">
+        <v>1256</v>
+      </c>
+      <c r="C504" t="s">
+        <v>286</v>
+      </c>
+      <c r="D504" t="s">
+        <v>1269</v>
+      </c>
+      <c r="E504" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="505" spans="1:5">
+      <c r="A505" t="s">
+        <v>1259</v>
+      </c>
+      <c r="B505" t="s">
+        <v>1258</v>
+      </c>
+      <c r="C505" t="s">
+        <v>286</v>
+      </c>
+      <c r="D505" t="s">
+        <v>1270</v>
+      </c>
+      <c r="E505" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="506" spans="1:5">
+      <c r="A506" t="s">
+        <v>568</v>
+      </c>
+      <c r="B506" t="s">
+        <v>569</v>
+      </c>
+      <c r="C506" t="s">
+        <v>286</v>
+      </c>
+      <c r="D506" t="s">
+        <v>570</v>
+      </c>
+      <c r="E506" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="507" spans="1:5">
+      <c r="A507" t="s">
+        <v>1260</v>
+      </c>
+      <c r="B507" t="s">
+        <v>572</v>
+      </c>
+      <c r="C507" t="s">
+        <v>286</v>
+      </c>
+      <c r="D507" t="s">
+        <v>573</v>
+      </c>
+      <c r="E507" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="508" spans="1:5">
+      <c r="A508" t="s">
+        <v>1261</v>
+      </c>
+      <c r="B508" t="s">
+        <v>575</v>
+      </c>
+      <c r="C508" t="s">
+        <v>286</v>
+      </c>
+      <c r="D508" t="s">
+        <v>576</v>
+      </c>
+      <c r="E508" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="509" spans="1:5">
+      <c r="A509" t="s">
+        <v>1262</v>
+      </c>
+      <c r="B509" t="s">
+        <v>578</v>
+      </c>
+      <c r="C509" t="s">
+        <v>286</v>
+      </c>
+      <c r="D509" t="s">
+        <v>579</v>
+      </c>
+      <c r="E509" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="510" spans="1:5">
+      <c r="A510" t="s">
+        <v>1264</v>
+      </c>
+      <c r="B510" t="s">
+        <v>1263</v>
+      </c>
+      <c r="C510" t="s">
+        <v>286</v>
+      </c>
+      <c r="D510" t="s">
+        <v>1271</v>
+      </c>
+      <c r="E510" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="511" spans="1:5">
+      <c r="A511" t="s">
+        <v>1266</v>
+      </c>
+      <c r="B511" t="s">
+        <v>1265</v>
+      </c>
+      <c r="C511" t="s">
+        <v>286</v>
+      </c>
+      <c r="D511" t="s">
+        <v>1272</v>
+      </c>
+      <c r="E511" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="512" spans="1:5">
+      <c r="A512" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B512" t="s">
+        <v>1273</v>
+      </c>
+      <c r="C512" t="s">
+        <v>725</v>
+      </c>
+      <c r="D512" t="s">
+        <v>734</v>
+      </c>
+      <c r="E512" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="513" spans="1:5">
+      <c r="A513" t="s">
+        <v>1276</v>
+      </c>
+      <c r="B513" t="s">
+        <v>1275</v>
+      </c>
+      <c r="C513" t="s">
+        <v>725</v>
+      </c>
+      <c r="D513" t="s">
+        <v>734</v>
+      </c>
+      <c r="E513" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="514" spans="1:5">
+      <c r="A514" t="s">
+        <v>1277</v>
+      </c>
+      <c r="B514" t="s">
+        <v>1278</v>
+      </c>
+      <c r="C514" t="s">
+        <v>725</v>
+      </c>
+      <c r="D514" t="s">
+        <v>734</v>
+      </c>
+      <c r="E514" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="515" spans="1:5">
+      <c r="A515" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B515" t="s">
+        <v>1279</v>
+      </c>
+      <c r="C515" t="s">
+        <v>725</v>
+      </c>
+      <c r="D515" t="s">
+        <v>734</v>
+      </c>
+      <c r="E515" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="516" spans="1:5">
+      <c r="A516" t="s">
+        <v>1285</v>
+      </c>
+      <c r="B516" t="s">
+        <v>1280</v>
+      </c>
+      <c r="C516" t="s">
+        <v>725</v>
+      </c>
+      <c r="D516" t="s">
+        <v>734</v>
+      </c>
+      <c r="E516" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="517" spans="1:5">
+      <c r="A517" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B517" t="s">
+        <v>1281</v>
+      </c>
+      <c r="C517" t="s">
+        <v>725</v>
+      </c>
+      <c r="D517" t="s">
+        <v>734</v>
+      </c>
+      <c r="E517" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="518" spans="1:5">
+      <c r="A518" t="s">
+        <v>1284</v>
+      </c>
+      <c r="B518" t="s">
+        <v>1282</v>
+      </c>
+      <c r="C518" t="s">
+        <v>725</v>
+      </c>
+      <c r="D518" t="s">
+        <v>734</v>
+      </c>
+      <c r="E518" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="519" spans="1:5">
+      <c r="A519" t="s">
+        <v>1288</v>
+      </c>
+      <c r="B519" t="s">
+        <v>1287</v>
+      </c>
+      <c r="C519" t="s">
+        <v>725</v>
+      </c>
+      <c r="D519" t="s">
+        <v>734</v>
+      </c>
+      <c r="E519" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="520" spans="1:5">
+      <c r="A520" t="s">
+        <v>1290</v>
+      </c>
+      <c r="B520" t="s">
+        <v>1289</v>
+      </c>
+      <c r="C520" t="s">
+        <v>725</v>
+      </c>
+      <c r="D520" t="s">
+        <v>734</v>
+      </c>
+      <c r="E520" t="s">
+        <v>734</v>
+      </c>
+    </row>
+    <row r="521" spans="1:5">
+      <c r="A521" t="s">
+        <v>1292</v>
+      </c>
+      <c r="B521" t="s">
+        <v>1291</v>
+      </c>
+      <c r="C521" t="s">
+        <v>725</v>
+      </c>
+      <c r="D521" t="s">
+        <v>734</v>
+      </c>
+      <c r="E521" t="s">
+        <v>734</v>
       </c>
     </row>
   </sheetData>

</xml_diff>